<commit_message>
Fill in main sheet with demo data
</commit_message>
<xml_diff>
--- a/waybills-creation/waybills-demo.xlsx
+++ b/waybills-creation/waybills-demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alinaaleks\Downloads\GitHub\automations\waybills-creation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB67728-568D-46BE-9B29-21DBD867D5D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3AA6F3-D4F4-4F4F-B232-78519BAA274C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="229">
   <si>
     <t>Типовая межотраслевая форма № СП-31</t>
   </si>
@@ -473,6 +473,9 @@
     <t>Таксировщик</t>
   </si>
   <si>
+    <t>Декларация соответствия</t>
+  </si>
+  <si>
     <t>id</t>
   </si>
   <si>
@@ -540,13 +543,232 @@
   </si>
   <si>
     <t>дата</t>
+  </si>
+  <si>
+    <t>9512</t>
+  </si>
+  <si>
+    <t>9513</t>
+  </si>
+  <si>
+    <t>9514</t>
+  </si>
+  <si>
+    <t>9515</t>
+  </si>
+  <si>
+    <t>9516</t>
+  </si>
+  <si>
+    <t>9517</t>
+  </si>
+  <si>
+    <t>9518</t>
+  </si>
+  <si>
+    <t>9519</t>
+  </si>
+  <si>
+    <t>9520</t>
+  </si>
+  <si>
+    <t>9521</t>
+  </si>
+  <si>
+    <t>ООО "АБВ"</t>
+  </si>
+  <si>
+    <t>КАМАЗ</t>
+  </si>
+  <si>
+    <t>МАЗ</t>
+  </si>
+  <si>
+    <t>Мерседес</t>
+  </si>
+  <si>
+    <t>Вольво</t>
+  </si>
+  <si>
+    <t>О975ВВ761</t>
+  </si>
+  <si>
+    <t>СК214461</t>
+  </si>
+  <si>
+    <t>А123МР777</t>
+  </si>
+  <si>
+    <t>ВЕ547391</t>
+  </si>
+  <si>
+    <t>М456ЕХ163</t>
+  </si>
+  <si>
+    <t>РТ932854</t>
+  </si>
+  <si>
+    <t>Т789АН402</t>
+  </si>
+  <si>
+    <t>МН678912</t>
+  </si>
+  <si>
+    <t>В321ОО599</t>
+  </si>
+  <si>
+    <t>АП456782</t>
+  </si>
+  <si>
+    <t>К654РМ750</t>
+  </si>
+  <si>
+    <t>ЕС327109</t>
+  </si>
+  <si>
+    <t>Н987НН222</t>
+  </si>
+  <si>
+    <t>ТР894567</t>
+  </si>
+  <si>
+    <t>С246ЕТ888</t>
+  </si>
+  <si>
+    <t>ОК213478</t>
+  </si>
+  <si>
+    <t>Р135РТ311</t>
+  </si>
+  <si>
+    <t>КМ765981</t>
+  </si>
+  <si>
+    <t>У864УН049</t>
+  </si>
+  <si>
+    <t>СХ432156</t>
+  </si>
+  <si>
+    <t>ООО "УФХ"</t>
+  </si>
+  <si>
+    <t>водитель_фио_полное</t>
+  </si>
+  <si>
+    <t>Водитель 1</t>
+  </si>
+  <si>
+    <t>Водитель 2</t>
+  </si>
+  <si>
+    <t>Водитель 3</t>
+  </si>
+  <si>
+    <t>Водитель 4</t>
+  </si>
+  <si>
+    <t>Водитель 5</t>
+  </si>
+  <si>
+    <t>Водитель 6</t>
+  </si>
+  <si>
+    <t>Водитель 7</t>
+  </si>
+  <si>
+    <t>Водитель 8</t>
+  </si>
+  <si>
+    <t>Водитель 9</t>
+  </si>
+  <si>
+    <t>Водитель 10</t>
+  </si>
+  <si>
+    <t>Краснодарский край</t>
+  </si>
+  <si>
+    <t>ИП ВГД</t>
+  </si>
+  <si>
+    <t>Ростовская обл.</t>
+  </si>
+  <si>
+    <t>пшеница</t>
+  </si>
+  <si>
+    <t>директор</t>
+  </si>
+  <si>
+    <t>Директор 1</t>
+  </si>
+  <si>
+    <t>Директор 2</t>
+  </si>
+  <si>
+    <t>Директор 3</t>
+  </si>
+  <si>
+    <t>Директор 4</t>
+  </si>
+  <si>
+    <t>Директор 5</t>
+  </si>
+  <si>
+    <t>Директор 6</t>
+  </si>
+  <si>
+    <t>Директор 7</t>
+  </si>
+  <si>
+    <t>Директор 8</t>
+  </si>
+  <si>
+    <t>Директор 9</t>
+  </si>
+  <si>
+    <t>Директор 10</t>
+  </si>
+  <si>
+    <t>кладовщик</t>
+  </si>
+  <si>
+    <t>Кладовщик 1</t>
+  </si>
+  <si>
+    <t>Кладовщик 2</t>
+  </si>
+  <si>
+    <t>Кладовщик 3</t>
+  </si>
+  <si>
+    <t>Кладовщик 4</t>
+  </si>
+  <si>
+    <t>Кладовщик 5</t>
+  </si>
+  <si>
+    <t>Кладовщик 6</t>
+  </si>
+  <si>
+    <t>Кладовщик 7</t>
+  </si>
+  <si>
+    <t>Кладовщик 8</t>
+  </si>
+  <si>
+    <t>Кладовщик 9</t>
+  </si>
+  <si>
+    <t>Кладовщик 10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -610,6 +832,12 @@
       <family val="1"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1963,7 +2191,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="391">
+  <cellXfs count="394">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -3096,6 +3324,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3378,10 +3611,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AA19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="12.1796875" customWidth="1"/>
+    <col min="1" max="1" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7" customWidth="1"/>
+    <col min="4" max="4" width="5" customWidth="1"/>
+    <col min="6" max="6" width="4.6328125" customWidth="1"/>
+    <col min="7" max="7" width="11.453125" customWidth="1"/>
+    <col min="9" max="9" width="10.36328125" customWidth="1"/>
+    <col min="10" max="10" width="11.08984375" customWidth="1"/>
+    <col min="11" max="11" width="11.26953125" customWidth="1"/>
+    <col min="12" max="12" width="9.7265625" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" customWidth="1"/>
+    <col min="17" max="17" width="10.6328125" customWidth="1"/>
+    <col min="23" max="23" width="11.54296875" customWidth="1"/>
+    <col min="25" max="26" width="11.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.35">
@@ -3464,154 +3709,1002 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:27" s="390" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="390" t="s">
+    <row r="2" spans="1:27" s="393" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="393" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" s="393" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="393" t="s">
+        <v>134</v>
+      </c>
+      <c r="D2" s="393" t="s">
+        <v>135</v>
+      </c>
+      <c r="E2" s="393" t="s">
+        <v>136</v>
+      </c>
+      <c r="F2" s="393" t="s">
+        <v>137</v>
+      </c>
+      <c r="G2" s="393" t="s">
+        <v>138</v>
+      </c>
+      <c r="H2" s="393" t="s">
+        <v>139</v>
+      </c>
+      <c r="I2" s="393" t="s">
+        <v>140</v>
+      </c>
+      <c r="J2" s="393" t="s">
+        <v>141</v>
+      </c>
+      <c r="K2" s="393" t="s">
+        <v>192</v>
+      </c>
+      <c r="L2" s="393" t="s">
+        <v>142</v>
+      </c>
+      <c r="M2" s="393" t="s">
+        <v>143</v>
+      </c>
+      <c r="N2" s="393" t="s">
+        <v>144</v>
+      </c>
+      <c r="O2" s="393" t="s">
+        <v>145</v>
+      </c>
+      <c r="P2" s="393" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q2" s="393" t="s">
+        <v>147</v>
+      </c>
+      <c r="R2" s="393" t="s">
+        <v>148</v>
+      </c>
+      <c r="S2" s="393" t="s">
+        <v>49</v>
+      </c>
+      <c r="T2" s="393" t="s">
+        <v>50</v>
+      </c>
+      <c r="U2" s="393" t="s">
+        <v>51</v>
+      </c>
+      <c r="V2" s="393" t="s">
+        <v>149</v>
+      </c>
+      <c r="W2" s="393" t="s">
+        <v>150</v>
+      </c>
+      <c r="X2" s="393" t="s">
+        <v>151</v>
+      </c>
+      <c r="Y2" s="393" t="s">
+        <v>152</v>
+      </c>
+      <c r="Z2" s="393" t="s">
+        <v>153</v>
+      </c>
+      <c r="AA2" s="393" t="s">
         <v>154</v>
-      </c>
-      <c r="B2" s="390" t="s">
-        <v>132</v>
-      </c>
-      <c r="C2" s="390" t="s">
-        <v>133</v>
-      </c>
-      <c r="D2" s="390" t="s">
-        <v>134</v>
-      </c>
-      <c r="E2" s="390" t="s">
-        <v>135</v>
-      </c>
-      <c r="F2" s="390" t="s">
-        <v>136</v>
-      </c>
-      <c r="G2" s="390" t="s">
-        <v>137</v>
-      </c>
-      <c r="H2" s="390" t="s">
-        <v>138</v>
-      </c>
-      <c r="I2" s="390" t="s">
-        <v>139</v>
-      </c>
-      <c r="J2" s="390" t="s">
-        <v>140</v>
-      </c>
-      <c r="K2" s="390" t="s">
-        <v>76</v>
-      </c>
-      <c r="L2" s="390" t="s">
-        <v>141</v>
-      </c>
-      <c r="M2" s="390" t="s">
-        <v>142</v>
-      </c>
-      <c r="N2" s="390" t="s">
-        <v>143</v>
-      </c>
-      <c r="O2" s="390" t="s">
-        <v>144</v>
-      </c>
-      <c r="P2" s="390" t="s">
-        <v>145</v>
-      </c>
-      <c r="Q2" s="390" t="s">
-        <v>146</v>
-      </c>
-      <c r="R2" s="390" t="s">
-        <v>147</v>
-      </c>
-      <c r="S2" s="390" t="s">
-        <v>49</v>
-      </c>
-      <c r="T2" s="390" t="s">
-        <v>50</v>
-      </c>
-      <c r="U2" s="390" t="s">
-        <v>51</v>
-      </c>
-      <c r="V2" s="390" t="s">
-        <v>148</v>
-      </c>
-      <c r="W2" s="390" t="s">
-        <v>149</v>
-      </c>
-      <c r="X2" s="390" t="s">
-        <v>150</v>
-      </c>
-      <c r="Y2" s="390" t="s">
-        <v>151</v>
-      </c>
-      <c r="Z2" s="390" t="s">
-        <v>152</v>
-      </c>
-      <c r="AA2" s="390" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A3" s="392">
+        <v>45915</v>
+      </c>
       <c r="B3">
         <v>1</v>
       </c>
+      <c r="C3" s="391" t="s">
+        <v>156</v>
+      </c>
+      <c r="D3">
+        <f>DAY(A3)</f>
+        <v>15</v>
+      </c>
+      <c r="E3" t="str">
+        <f>CHOOSE(MONTH(A3),"января","февраля","марта","апреля","мая","июня","июля","августа","сентября","октября","ноября","декабря")</f>
+        <v>сентября</v>
+      </c>
+      <c r="F3">
+        <f>MOD(YEAR(A3),100)</f>
+        <v>25</v>
+      </c>
+      <c r="G3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H3" t="s">
+        <v>167</v>
+      </c>
+      <c r="I3" t="s">
+        <v>171</v>
+      </c>
+      <c r="J3" t="s">
+        <v>204</v>
+      </c>
+      <c r="K3" t="s">
+        <v>193</v>
+      </c>
+      <c r="L3" t="str">
+        <f>G3</f>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="M3" t="s">
+        <v>191</v>
+      </c>
+      <c r="N3" t="s">
+        <v>203</v>
+      </c>
+      <c r="O3" t="str">
+        <f>G3</f>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="P3" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>172</v>
+      </c>
+      <c r="R3" t="s">
+        <v>206</v>
+      </c>
+      <c r="S3">
+        <v>34600</v>
+      </c>
+      <c r="T3">
+        <v>15220</v>
+      </c>
+      <c r="U3">
+        <v>19380</v>
+      </c>
+      <c r="V3" t="s">
+        <v>207</v>
+      </c>
+      <c r="W3" t="s">
+        <v>208</v>
+      </c>
+      <c r="X3" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>219</v>
+      </c>
+      <c r="Z3" t="str">
+        <f>K3</f>
+        <v>Водитель 1</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A4" s="392">
+        <v>45915</v>
+      </c>
       <c r="B4">
         <v>2</v>
       </c>
+      <c r="C4" s="391" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4">
+        <f t="shared" ref="D4:D12" si="0">DAY(A4)</f>
+        <v>15</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" ref="E4:E12" si="1">CHOOSE(MONTH(A4),"января","февраля","марта","апреля","мая","июня","июля","августа","сентября","октября","ноября","декабря")</f>
+        <v>сентября</v>
+      </c>
+      <c r="F4">
+        <f t="shared" ref="F4:F12" si="2">MOD(YEAR(A4),100)</f>
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>166</v>
+      </c>
+      <c r="H4" t="s">
+        <v>167</v>
+      </c>
+      <c r="I4" t="s">
+        <v>173</v>
+      </c>
+      <c r="J4" t="s">
+        <v>204</v>
+      </c>
+      <c r="K4" t="s">
+        <v>194</v>
+      </c>
+      <c r="L4" t="str">
+        <f t="shared" ref="L4:L12" si="3">G4</f>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="M4" t="s">
+        <v>191</v>
+      </c>
+      <c r="N4" t="s">
+        <v>203</v>
+      </c>
+      <c r="O4" t="str">
+        <f t="shared" ref="O4:O12" si="4">G4</f>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="P4" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>174</v>
+      </c>
+      <c r="R4" t="s">
+        <v>206</v>
+      </c>
+      <c r="S4">
+        <v>35120</v>
+      </c>
+      <c r="T4">
+        <v>14850</v>
+      </c>
+      <c r="U4">
+        <v>20270</v>
+      </c>
+      <c r="V4" t="s">
+        <v>207</v>
+      </c>
+      <c r="W4" t="s">
+        <v>209</v>
+      </c>
+      <c r="X4" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>220</v>
+      </c>
+      <c r="Z4" t="str">
+        <f t="shared" ref="Z4:Z12" si="5">K4</f>
+        <v>Водитель 2</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A5" s="392">
+        <v>45915</v>
+      </c>
       <c r="B5">
         <v>3</v>
       </c>
+      <c r="C5" s="391" t="s">
+        <v>158</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="1"/>
+        <v>сентября</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="2"/>
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>166</v>
+      </c>
+      <c r="H5" t="s">
+        <v>168</v>
+      </c>
+      <c r="I5" t="s">
+        <v>175</v>
+      </c>
+      <c r="J5" t="s">
+        <v>204</v>
+      </c>
+      <c r="K5" t="s">
+        <v>195</v>
+      </c>
+      <c r="L5" t="str">
+        <f t="shared" si="3"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="M5" t="s">
+        <v>191</v>
+      </c>
+      <c r="N5" t="s">
+        <v>203</v>
+      </c>
+      <c r="O5" t="str">
+        <f t="shared" si="4"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="P5" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>176</v>
+      </c>
+      <c r="R5" t="s">
+        <v>206</v>
+      </c>
+      <c r="S5">
+        <v>33890</v>
+      </c>
+      <c r="T5">
+        <v>15640</v>
+      </c>
+      <c r="U5">
+        <v>18250</v>
+      </c>
+      <c r="V5" t="s">
+        <v>207</v>
+      </c>
+      <c r="W5" t="s">
+        <v>210</v>
+      </c>
+      <c r="X5" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>221</v>
+      </c>
+      <c r="Z5" t="str">
+        <f t="shared" si="5"/>
+        <v>Водитель 3</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A6" s="392">
+        <v>45950</v>
+      </c>
       <c r="B6">
         <v>4</v>
       </c>
+      <c r="C6" s="391" t="s">
+        <v>159</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="1"/>
+        <v>октября</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="2"/>
+        <v>25</v>
+      </c>
+      <c r="G6" t="s">
+        <v>166</v>
+      </c>
+      <c r="H6" t="s">
+        <v>169</v>
+      </c>
+      <c r="I6" t="s">
+        <v>177</v>
+      </c>
+      <c r="J6" t="s">
+        <v>204</v>
+      </c>
+      <c r="K6" t="s">
+        <v>196</v>
+      </c>
+      <c r="L6" t="str">
+        <f t="shared" si="3"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="M6" t="s">
+        <v>191</v>
+      </c>
+      <c r="N6" t="s">
+        <v>203</v>
+      </c>
+      <c r="O6" t="str">
+        <f t="shared" si="4"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="P6" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>178</v>
+      </c>
+      <c r="R6" t="s">
+        <v>206</v>
+      </c>
+      <c r="S6">
+        <v>35980</v>
+      </c>
+      <c r="T6">
+        <v>14320</v>
+      </c>
+      <c r="U6">
+        <v>21660</v>
+      </c>
+      <c r="V6" t="s">
+        <v>207</v>
+      </c>
+      <c r="W6" t="s">
+        <v>211</v>
+      </c>
+      <c r="X6" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>222</v>
+      </c>
+      <c r="Z6" t="str">
+        <f t="shared" si="5"/>
+        <v>Водитель 4</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>132</v>
+      </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:27" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="392">
+        <v>45951</v>
+      </c>
       <c r="B7">
         <v>5</v>
       </c>
-      <c r="G7" s="390"/>
-      <c r="H7" s="390"/>
-      <c r="I7" s="390"/>
-      <c r="J7" s="390"/>
-      <c r="K7" s="390"/>
-      <c r="L7" s="390"/>
-      <c r="M7" s="390"/>
-      <c r="N7" s="390"/>
-      <c r="O7" s="390"/>
-      <c r="P7" s="390"/>
-      <c r="Q7" s="390"/>
-      <c r="R7" s="390"/>
-      <c r="S7" s="390"/>
-      <c r="T7" s="390"/>
+      <c r="C7" s="391" t="s">
+        <v>160</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="E7" t="str">
+        <f t="shared" si="1"/>
+        <v>октября</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="2"/>
+        <v>25</v>
+      </c>
+      <c r="G7" t="s">
+        <v>166</v>
+      </c>
+      <c r="H7" t="s">
+        <v>167</v>
+      </c>
+      <c r="I7" s="390" t="s">
+        <v>179</v>
+      </c>
+      <c r="J7" t="s">
+        <v>204</v>
+      </c>
+      <c r="K7" t="s">
+        <v>197</v>
+      </c>
+      <c r="L7" t="str">
+        <f t="shared" si="3"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="M7" t="s">
+        <v>191</v>
+      </c>
+      <c r="N7" t="s">
+        <v>203</v>
+      </c>
+      <c r="O7" t="str">
+        <f t="shared" si="4"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="P7" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q7" s="390" t="s">
+        <v>180</v>
+      </c>
+      <c r="R7" t="s">
+        <v>206</v>
+      </c>
+      <c r="S7" s="390">
+        <v>32750</v>
+      </c>
+      <c r="T7" s="390">
+        <v>15910</v>
+      </c>
+      <c r="U7">
+        <v>16840</v>
+      </c>
+      <c r="V7" t="s">
+        <v>207</v>
+      </c>
+      <c r="W7" t="s">
+        <v>212</v>
+      </c>
+      <c r="X7" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>223</v>
+      </c>
+      <c r="Z7" t="str">
+        <f t="shared" si="5"/>
+        <v>Водитель 5</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A8" s="392">
+        <v>45952</v>
+      </c>
       <c r="B8">
         <v>6</v>
       </c>
+      <c r="C8" s="391" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" si="1"/>
+        <v>октября</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="2"/>
+        <v>25</v>
+      </c>
+      <c r="G8" t="s">
+        <v>166</v>
+      </c>
+      <c r="H8" t="s">
+        <v>167</v>
+      </c>
+      <c r="I8" t="s">
+        <v>181</v>
+      </c>
+      <c r="J8" t="s">
+        <v>204</v>
+      </c>
+      <c r="K8" t="s">
+        <v>198</v>
+      </c>
+      <c r="L8" t="str">
+        <f t="shared" si="3"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="M8" t="s">
+        <v>191</v>
+      </c>
+      <c r="N8" t="s">
+        <v>203</v>
+      </c>
+      <c r="O8" t="str">
+        <f t="shared" si="4"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="P8" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>182</v>
+      </c>
+      <c r="R8" t="s">
+        <v>206</v>
+      </c>
+      <c r="S8">
+        <v>34410</v>
+      </c>
+      <c r="T8">
+        <v>15180</v>
+      </c>
+      <c r="U8">
+        <v>19230</v>
+      </c>
+      <c r="V8" t="s">
+        <v>207</v>
+      </c>
+      <c r="W8" t="s">
+        <v>213</v>
+      </c>
+      <c r="X8" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>224</v>
+      </c>
+      <c r="Z8" t="str">
+        <f t="shared" si="5"/>
+        <v>Водитель 6</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A9" s="392">
+        <v>46000</v>
+      </c>
       <c r="B9">
         <v>7</v>
       </c>
+      <c r="C9" s="391" t="s">
+        <v>162</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="1"/>
+        <v>декабря</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="2"/>
+        <v>25</v>
+      </c>
+      <c r="G9" t="s">
+        <v>166</v>
+      </c>
+      <c r="H9" t="s">
+        <v>168</v>
+      </c>
+      <c r="I9" t="s">
+        <v>183</v>
+      </c>
+      <c r="J9" t="s">
+        <v>204</v>
+      </c>
+      <c r="K9" t="s">
+        <v>199</v>
+      </c>
+      <c r="L9" t="str">
+        <f t="shared" si="3"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="M9" t="s">
+        <v>191</v>
+      </c>
+      <c r="N9" t="s">
+        <v>203</v>
+      </c>
+      <c r="O9" t="str">
+        <f t="shared" si="4"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="P9" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>184</v>
+      </c>
+      <c r="R9" t="s">
+        <v>206</v>
+      </c>
+      <c r="S9">
+        <v>35560</v>
+      </c>
+      <c r="T9">
+        <v>14790</v>
+      </c>
+      <c r="U9">
+        <v>20770</v>
+      </c>
+      <c r="V9" t="s">
+        <v>207</v>
+      </c>
+      <c r="W9" t="s">
+        <v>214</v>
+      </c>
+      <c r="X9" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>225</v>
+      </c>
+      <c r="Z9" t="str">
+        <f t="shared" si="5"/>
+        <v>Водитель 7</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A10" s="392">
+        <v>46045</v>
+      </c>
       <c r="B10">
         <v>8</v>
       </c>
+      <c r="C10" s="391" t="s">
+        <v>163</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="1"/>
+        <v>января</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
+      <c r="G10" t="s">
+        <v>166</v>
+      </c>
+      <c r="H10" t="s">
+        <v>169</v>
+      </c>
+      <c r="I10" t="s">
+        <v>185</v>
+      </c>
+      <c r="J10" t="s">
+        <v>204</v>
+      </c>
+      <c r="K10" t="s">
+        <v>200</v>
+      </c>
+      <c r="L10" t="str">
+        <f t="shared" si="3"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="M10" t="s">
+        <v>191</v>
+      </c>
+      <c r="N10" t="s">
+        <v>203</v>
+      </c>
+      <c r="O10" t="str">
+        <f t="shared" si="4"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="P10" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>186</v>
+      </c>
+      <c r="R10" t="s">
+        <v>206</v>
+      </c>
+      <c r="S10">
+        <v>33280</v>
+      </c>
+      <c r="T10">
+        <v>15460</v>
+      </c>
+      <c r="U10">
+        <v>17820</v>
+      </c>
+      <c r="V10" t="s">
+        <v>207</v>
+      </c>
+      <c r="W10" t="s">
+        <v>215</v>
+      </c>
+      <c r="X10" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>226</v>
+      </c>
+      <c r="Z10" t="str">
+        <f t="shared" si="5"/>
+        <v>Водитель 8</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A11" s="392">
+        <v>46083</v>
+      </c>
       <c r="B11">
         <v>9</v>
       </c>
+      <c r="C11" s="391" t="s">
+        <v>164</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="1"/>
+        <v>марта</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
+      <c r="G11" t="s">
+        <v>166</v>
+      </c>
+      <c r="H11" t="s">
+        <v>170</v>
+      </c>
+      <c r="I11" t="s">
+        <v>187</v>
+      </c>
+      <c r="J11" t="s">
+        <v>204</v>
+      </c>
+      <c r="K11" t="s">
+        <v>201</v>
+      </c>
+      <c r="L11" t="str">
+        <f t="shared" si="3"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="M11" t="s">
+        <v>191</v>
+      </c>
+      <c r="N11" t="s">
+        <v>203</v>
+      </c>
+      <c r="O11" t="str">
+        <f t="shared" si="4"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="P11" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>188</v>
+      </c>
+      <c r="R11" t="s">
+        <v>206</v>
+      </c>
+      <c r="S11">
+        <v>34870</v>
+      </c>
+      <c r="T11">
+        <v>14950</v>
+      </c>
+      <c r="U11">
+        <v>19920</v>
+      </c>
+      <c r="V11" t="s">
+        <v>207</v>
+      </c>
+      <c r="W11" t="s">
+        <v>216</v>
+      </c>
+      <c r="X11" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>227</v>
+      </c>
+      <c r="Z11" t="str">
+        <f t="shared" si="5"/>
+        <v>Водитель 9</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A12" s="392">
+        <v>46180</v>
+      </c>
       <c r="B12">
         <v>10</v>
       </c>
+      <c r="C12" s="391" t="s">
+        <v>165</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="1"/>
+        <v>июня</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
+      <c r="G12" t="s">
+        <v>166</v>
+      </c>
+      <c r="H12" t="s">
+        <v>170</v>
+      </c>
+      <c r="I12" t="s">
+        <v>189</v>
+      </c>
+      <c r="J12" t="s">
+        <v>204</v>
+      </c>
+      <c r="K12" t="s">
+        <v>202</v>
+      </c>
+      <c r="L12" t="str">
+        <f t="shared" si="3"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="M12" t="s">
+        <v>191</v>
+      </c>
+      <c r="N12" t="s">
+        <v>203</v>
+      </c>
+      <c r="O12" t="str">
+        <f t="shared" si="4"/>
+        <v>ООО "АБВ"</v>
+      </c>
+      <c r="P12" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>190</v>
+      </c>
+      <c r="R12" t="s">
+        <v>206</v>
+      </c>
+      <c r="S12">
+        <v>36240</v>
+      </c>
+      <c r="T12">
+        <v>14130</v>
+      </c>
+      <c r="U12">
+        <v>22110</v>
+      </c>
+      <c r="V12" t="s">
+        <v>207</v>
+      </c>
+      <c r="W12" t="s">
+        <v>217</v>
+      </c>
+      <c r="X12" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>228</v>
+      </c>
+      <c r="Z12" t="str">
+        <f t="shared" si="5"/>
+        <v>Водитель 10</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="C13" s="391"/>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="C14" s="391"/>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="C15" s="391"/>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="C16" s="391"/>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C17" s="391"/>
+    </row>
+    <row r="18" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C18" s="391"/>
+    </row>
+    <row r="19" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C19" s="391"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3631,7 +4724,7 @@
         <v>0</v>
       </c>
       <c r="DE1" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="2:109" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Change demo data to more realistic, yet still synthetic
</commit_message>
<xml_diff>
--- a/waybills-creation/waybills-demo.xlsx
+++ b/waybills-creation/waybills-demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alinaaleks\Downloads\GitHub\automations\waybills-creation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D23071-C1CA-48F0-BF13-DD902D5E152A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3683B0E0-DDE5-48C1-BEA4-619DE8D5444B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="258">
   <si>
     <t>Типовая межотраслевая форма № СП-31</t>
   </si>
@@ -521,21 +521,12 @@
     <t>продукция</t>
   </si>
   <si>
-    <t>отпуск_должность</t>
-  </si>
-  <si>
-    <t>отпуск_фио</t>
-  </si>
-  <si>
     <t>сдал_должность</t>
   </si>
   <si>
     <t>сдал_фио</t>
   </si>
   <si>
-    <t>принял_фио</t>
-  </si>
-  <si>
     <t>приложение</t>
   </si>
   <si>
@@ -572,9 +563,6 @@
     <t>9521</t>
   </si>
   <si>
-    <t>ООО "АБВ"</t>
-  </si>
-  <si>
     <t>ВЕ547391</t>
   </si>
   <si>
@@ -602,48 +590,12 @@
     <t>СХ432156</t>
   </si>
   <si>
-    <t>ООО "УФХ"</t>
-  </si>
-  <si>
-    <t>водитель_фио_полное</t>
-  </si>
-  <si>
-    <t>Водитель 1</t>
-  </si>
-  <si>
-    <t>Водитель 2</t>
-  </si>
-  <si>
-    <t>Водитель 3</t>
-  </si>
-  <si>
-    <t>Водитель 4</t>
-  </si>
-  <si>
-    <t>Водитель 5</t>
-  </si>
-  <si>
-    <t>Водитель 6</t>
-  </si>
-  <si>
-    <t>Водитель 7</t>
-  </si>
-  <si>
-    <t>Водитель 8</t>
-  </si>
-  <si>
-    <t>Водитель 9</t>
-  </si>
-  <si>
-    <t>Водитель 10</t>
+    <t>водитель_фио</t>
   </si>
   <si>
     <t>Краснодарский край</t>
   </si>
   <si>
-    <t>ИП ВГД</t>
-  </si>
-  <si>
     <t>Ростовская обл.</t>
   </si>
   <si>
@@ -653,69 +605,9 @@
     <t>директор</t>
   </si>
   <si>
-    <t>Директор 1</t>
-  </si>
-  <si>
-    <t>Директор 2</t>
-  </si>
-  <si>
-    <t>Директор 3</t>
-  </si>
-  <si>
-    <t>Директор 4</t>
-  </si>
-  <si>
-    <t>Директор 5</t>
-  </si>
-  <si>
-    <t>Директор 6</t>
-  </si>
-  <si>
-    <t>Директор 7</t>
-  </si>
-  <si>
-    <t>Директор 8</t>
-  </si>
-  <si>
-    <t>Директор 9</t>
-  </si>
-  <si>
-    <t>Директор 10</t>
-  </si>
-  <si>
     <t>кладовщик</t>
   </si>
   <si>
-    <t>Кладовщик 1</t>
-  </si>
-  <si>
-    <t>Кладовщик 2</t>
-  </si>
-  <si>
-    <t>Кладовщик 3</t>
-  </si>
-  <si>
-    <t>Кладовщик 4</t>
-  </si>
-  <si>
-    <t>Кладовщик 5</t>
-  </si>
-  <si>
-    <t>Кладовщик 6</t>
-  </si>
-  <si>
-    <t>Кладовщик 7</t>
-  </si>
-  <si>
-    <t>Кладовщик 8</t>
-  </si>
-  <si>
-    <t>Кладовщик 9</t>
-  </si>
-  <si>
-    <t>Кладовщик 10</t>
-  </si>
-  <si>
     <t>гос_номер-авто</t>
   </si>
   <si>
@@ -756,6 +648,207 @@
   </si>
   <si>
     <t>данные для вставки</t>
+  </si>
+  <si>
+    <t>отпустил_должность</t>
+  </si>
+  <si>
+    <t>отпустил_фио</t>
+  </si>
+  <si>
+    <t>ячмень</t>
+  </si>
+  <si>
+    <t>пшеница 3 класса</t>
+  </si>
+  <si>
+    <t>кукуруза</t>
+  </si>
+  <si>
+    <t>Ставропольский край</t>
+  </si>
+  <si>
+    <t>Таргин Алексей Викторович</t>
+  </si>
+  <si>
+    <t>Моргин Павел Сергеевич</t>
+  </si>
+  <si>
+    <t>Калевин Денис Игоревич</t>
+  </si>
+  <si>
+    <t>Родевский Андрей Николаевич</t>
+  </si>
+  <si>
+    <t>Семиров Артём Викторович</t>
+  </si>
+  <si>
+    <t>Горевин Максим Олегович</t>
+  </si>
+  <si>
+    <t>Даневский Кирилл Андреевич</t>
+  </si>
+  <si>
+    <t>Лемиров Сергей Андреевич</t>
+  </si>
+  <si>
+    <t>Неворин Дмитрий Олегович</t>
+  </si>
+  <si>
+    <t>Заревский Павел Николаевич</t>
+  </si>
+  <si>
+    <t>Иванор Сергей Петрович</t>
+  </si>
+  <si>
+    <t>Смирев Андрей Николаевич</t>
+  </si>
+  <si>
+    <t>Кузнецын Алексей Викторович</t>
+  </si>
+  <si>
+    <t>Попович Денис Олегович</t>
+  </si>
+  <si>
+    <t>Волягин Егор Дмитриевич</t>
+  </si>
+  <si>
+    <t>Крестовин Роман Алексеевич</t>
+  </si>
+  <si>
+    <t>Орлинов Виктор Павлович</t>
+  </si>
+  <si>
+    <t>Белярев Кирилл Сергеевич</t>
+  </si>
+  <si>
+    <t>Снегиров Андрей Олегович</t>
+  </si>
+  <si>
+    <t>Ветровин Денис Игоревич</t>
+  </si>
+  <si>
+    <t>ООО "АгроФлоу X1"</t>
+  </si>
+  <si>
+    <t>ООО "ЗерноПриём 24A"</t>
+  </si>
+  <si>
+    <t>ООО "ГрейнПорт-Х"</t>
+  </si>
+  <si>
+    <t>ООО "АгроЛогистик Z7"</t>
+  </si>
+  <si>
+    <t>ООО "ЮгЗерноСнаб X2"</t>
+  </si>
+  <si>
+    <t>ООО "ПотокАгро Q1"</t>
+  </si>
+  <si>
+    <t>ООО "ТерраГрейн 9X"</t>
+  </si>
+  <si>
+    <t>ООО "ФермаТрейд-Х"</t>
+  </si>
+  <si>
+    <t>ООО "ЗерноХаб 17B"</t>
+  </si>
+  <si>
+    <t>ООО "АгроСклад V3"</t>
+  </si>
+  <si>
+    <t>ООО "АгроЭкспорт X9"</t>
+  </si>
+  <si>
+    <t>ООО "ЗерноОтгрузка 21A"</t>
+  </si>
+  <si>
+    <t>ООО "ТрансАгроЛиния-Х"</t>
+  </si>
+  <si>
+    <t>ООО "ЮгПоставка Q8"</t>
+  </si>
+  <si>
+    <t>ООО "ГрейнСинтез 3X"</t>
+  </si>
+  <si>
+    <t>ООО "АгроВектор Z2"</t>
+  </si>
+  <si>
+    <t>ООО "ПоляТрейд X5"</t>
+  </si>
+  <si>
+    <t>ООО "ЗерноЛайн-24B"</t>
+  </si>
+  <si>
+    <t>ООО "ФлоуАгро V1"</t>
+  </si>
+  <si>
+    <t>ООО "АгроТерминал X7"</t>
+  </si>
+  <si>
+    <t>ООО "ТрансВектор X1"</t>
+  </si>
+  <si>
+    <t>ООО "ГрузЛогистика 14A"</t>
+  </si>
+  <si>
+    <t>ООО "АвтоЗерноПоток-Х"</t>
+  </si>
+  <si>
+    <t>ООО "ЮгТрансСистема Q3"</t>
+  </si>
+  <si>
+    <t>ООО "ГрейнТрансЛайн X8"</t>
+  </si>
+  <si>
+    <t>ООО "АгроАвтоСинтез 6B"</t>
+  </si>
+  <si>
+    <t>ООО "ДорТрансАгро X2"</t>
+  </si>
+  <si>
+    <t>ООО "ЛогистикФлоу 19X"</t>
+  </si>
+  <si>
+    <t>ООО "ЗерноМобиль V4"</t>
+  </si>
+  <si>
+    <t>ООО "ТрансЮгЭкспресс X9"</t>
+  </si>
+  <si>
+    <t>принял_фио_сокр</t>
+  </si>
+  <si>
+    <t>Сидорина М.А.</t>
+  </si>
+  <si>
+    <t>Петровина О.С.</t>
+  </si>
+  <si>
+    <t>Калинина Н.В.</t>
+  </si>
+  <si>
+    <t>Горина Е.А.</t>
+  </si>
+  <si>
+    <t>Таревская И.О.</t>
+  </si>
+  <si>
+    <t>Карпелин М.А.</t>
+  </si>
+  <si>
+    <t>Новаров П.Н.</t>
+  </si>
+  <si>
+    <t>Сольцев А.В.</t>
+  </si>
+  <si>
+    <t>Ардентов И.С.</t>
+  </si>
+  <si>
+    <t>Родина В.А.</t>
   </si>
 </sst>
 </file>
@@ -833,7 +926,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -870,6 +963,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="106">
     <border>
@@ -2209,7 +2314,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="424">
+  <cellXfs count="430">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -3399,15 +3504,23 @@
     <xf numFmtId="3" fontId="2" fillId="6" borderId="72" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="72" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3716,11 +3829,11 @@
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A1" s="374" t="s">
-        <v>225</v>
+        <v>189</v>
       </c>
       <c r="B1" s="375"/>
       <c r="C1" s="384" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="D1" s="385"/>
       <c r="E1" s="385"/>
@@ -3832,10 +3945,10 @@
     </row>
     <row r="3" spans="1:28" s="373" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="378" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B3" s="379" t="s">
-        <v>224</v>
+        <v>188</v>
       </c>
       <c r="C3" s="388" t="s">
         <v>133</v>
@@ -3859,13 +3972,13 @@
         <v>139</v>
       </c>
       <c r="J3" s="391" t="s">
-        <v>213</v>
+        <v>177</v>
       </c>
       <c r="K3" s="389" t="s">
         <v>140</v>
       </c>
-      <c r="L3" s="389" t="s">
-        <v>176</v>
+      <c r="L3" s="423" t="s">
+        <v>171</v>
       </c>
       <c r="M3" s="389" t="s">
         <v>141</v>
@@ -3898,22 +4011,22 @@
         <v>51</v>
       </c>
       <c r="W3" s="389" t="s">
+        <v>191</v>
+      </c>
+      <c r="X3" s="389" t="s">
+        <v>192</v>
+      </c>
+      <c r="Y3" s="389" t="s">
         <v>148</v>
       </c>
-      <c r="X3" s="389" t="s">
+      <c r="Z3" s="389" t="s">
         <v>149</v>
       </c>
-      <c r="Y3" s="389" t="s">
+      <c r="AA3" s="427" t="s">
+        <v>247</v>
+      </c>
+      <c r="AB3" s="392" t="s">
         <v>150</v>
-      </c>
-      <c r="Z3" s="389" t="s">
-        <v>151</v>
-      </c>
-      <c r="AA3" s="389" t="s">
-        <v>152</v>
-      </c>
-      <c r="AB3" s="392" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.35">
@@ -3921,13 +4034,13 @@
         <v>45915</v>
       </c>
       <c r="B4" s="381" t="s">
-        <v>214</v>
+        <v>178</v>
       </c>
       <c r="C4" s="376">
         <v>1</v>
       </c>
       <c r="D4" s="393" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E4" s="394">
         <f>DAY(A4)</f>
@@ -3942,7 +4055,7 @@
         <v>25</v>
       </c>
       <c r="H4" s="387" t="s">
-        <v>165</v>
+        <v>217</v>
       </c>
       <c r="I4" s="395" t="str">
         <f>LEFT(B4,FIND(" ",B4)-1)</f>
@@ -3953,34 +4066,34 @@
         <v>О975ВВ761</v>
       </c>
       <c r="K4" s="387" t="s">
-        <v>188</v>
-      </c>
-      <c r="L4" s="387" t="s">
-        <v>177</v>
+        <v>237</v>
+      </c>
+      <c r="L4" s="424" t="s">
+        <v>207</v>
       </c>
       <c r="M4" s="387" t="str">
         <f>H4</f>
-        <v>ООО "АБВ"</v>
+        <v>ООО "АгроФлоу X1"</v>
       </c>
       <c r="N4" s="387" t="s">
-        <v>175</v>
+        <v>227</v>
       </c>
       <c r="O4" s="387" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="P4" s="387" t="str">
         <f>H4</f>
-        <v>ООО "АБВ"</v>
+        <v>ООО "АгроФлоу X1"</v>
       </c>
       <c r="Q4" s="387" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="R4" s="395" t="str">
         <f>MID(B4,FIND(" ",B4,FIND(" ",B4)+1)+1,LEN(B4)-FIND(" ",B4,FIND(" ",B4)+1))</f>
         <v>СК214461</v>
       </c>
       <c r="S4" s="387" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="T4" s="387">
         <v>34600</v>
@@ -3992,20 +4105,22 @@
         <v>19380</v>
       </c>
       <c r="W4" s="387" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="X4" s="387" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="Y4" s="387" t="s">
-        <v>202</v>
+        <v>176</v>
       </c>
       <c r="Z4" s="387" t="s">
-        <v>203</v>
-      </c>
-      <c r="AA4" s="387" t="str">
-        <f>L4</f>
-        <v>Водитель 1</v>
+        <v>248</v>
+      </c>
+      <c r="AA4" s="428" t="str">
+        <f>LEFT(L4,FIND(" ",L4)-1) &amp; " " &amp;
+MID(L4,FIND(" ",L4)+1,1) &amp; "." &amp;
+MID(L4,FIND(" ",L4,FIND(" ",L4)+1)+1,1) &amp; "."</f>
+        <v>Иванор С.П.</v>
       </c>
       <c r="AB4" s="377" t="s">
         <v>132</v>
@@ -4016,13 +4131,13 @@
         <v>45915</v>
       </c>
       <c r="B5" s="381" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="C5" s="376">
         <v>2</v>
       </c>
       <c r="D5" s="393" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="E5" s="394">
         <f t="shared" ref="E5:E13" si="0">DAY(A5)</f>
@@ -4037,7 +4152,7 @@
         <v>25</v>
       </c>
       <c r="H5" s="387" t="s">
-        <v>165</v>
+        <v>218</v>
       </c>
       <c r="I5" s="395" t="str">
         <f t="shared" ref="I5:I12" si="3">LEFT(B5,FIND(" ",B5)-1)</f>
@@ -4048,33 +4163,33 @@
         <v>А123МР777</v>
       </c>
       <c r="K5" s="387" t="s">
-        <v>188</v>
-      </c>
-      <c r="L5" s="387" t="s">
-        <v>178</v>
+        <v>238</v>
+      </c>
+      <c r="L5" s="424" t="s">
+        <v>208</v>
       </c>
       <c r="M5" s="387" t="str">
         <f t="shared" ref="M5:M13" si="5">H5</f>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ЗерноПриём 24A"</v>
       </c>
       <c r="N5" s="387" t="s">
-        <v>175</v>
+        <v>228</v>
       </c>
       <c r="O5" s="387" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="P5" s="387" t="str">
         <f t="shared" ref="P5:P13" si="6">H5</f>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ЗерноПриём 24A"</v>
       </c>
       <c r="Q5" s="387" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="R5" s="395" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="S5" s="387" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="T5" s="387">
         <v>35120</v>
@@ -4086,20 +4201,22 @@
         <v>20270</v>
       </c>
       <c r="W5" s="387" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="X5" s="387" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="Y5" s="387" t="s">
-        <v>202</v>
+        <v>176</v>
       </c>
       <c r="Z5" s="387" t="s">
-        <v>204</v>
-      </c>
-      <c r="AA5" s="387" t="str">
-        <f t="shared" ref="AA5:AA13" si="7">L5</f>
-        <v>Водитель 2</v>
+        <v>249</v>
+      </c>
+      <c r="AA5" s="428" t="str">
+        <f t="shared" ref="AA5:AA13" si="7">LEFT(L5,FIND(" ",L5)-1) &amp; " " &amp;
+MID(L5,FIND(" ",L5)+1,1) &amp; "." &amp;
+MID(L5,FIND(" ",L5,FIND(" ",L5)+1)+1,1) &amp; "."</f>
+        <v>Смирев А.Н.</v>
       </c>
       <c r="AB5" s="377" t="s">
         <v>132</v>
@@ -4110,13 +4227,13 @@
         <v>45915</v>
       </c>
       <c r="B6" s="381" t="s">
-        <v>216</v>
+        <v>180</v>
       </c>
       <c r="C6" s="376">
         <v>3</v>
       </c>
       <c r="D6" s="393" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E6" s="394">
         <f t="shared" si="0"/>
@@ -4131,7 +4248,7 @@
         <v>25</v>
       </c>
       <c r="H6" s="387" t="s">
-        <v>165</v>
+        <v>219</v>
       </c>
       <c r="I6" s="395" t="str">
         <f t="shared" si="3"/>
@@ -4142,33 +4259,33 @@
         <v>М456ЕХ163</v>
       </c>
       <c r="K6" s="387" t="s">
-        <v>188</v>
-      </c>
-      <c r="L6" s="387" t="s">
-        <v>179</v>
+        <v>239</v>
+      </c>
+      <c r="L6" s="424" t="s">
+        <v>209</v>
       </c>
       <c r="M6" s="387" t="str">
         <f t="shared" si="5"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ГрейнПорт-Х"</v>
       </c>
       <c r="N6" s="387" t="s">
-        <v>175</v>
+        <v>229</v>
       </c>
       <c r="O6" s="387" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="P6" s="387" t="str">
         <f t="shared" si="6"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ГрейнПорт-Х"</v>
       </c>
       <c r="Q6" s="387" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="R6" s="395" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="S6" s="387" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="T6" s="387">
         <v>33890</v>
@@ -4180,20 +4297,20 @@
         <v>18250</v>
       </c>
       <c r="W6" s="387" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="X6" s="387" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="Y6" s="387" t="s">
-        <v>202</v>
+        <v>176</v>
       </c>
       <c r="Z6" s="387" t="s">
-        <v>205</v>
-      </c>
-      <c r="AA6" s="387" t="str">
+        <v>250</v>
+      </c>
+      <c r="AA6" s="428" t="str">
         <f t="shared" si="7"/>
-        <v>Водитель 3</v>
+        <v>Кузнецын А.В.</v>
       </c>
       <c r="AB6" s="377" t="s">
         <v>132</v>
@@ -4204,13 +4321,13 @@
         <v>45950</v>
       </c>
       <c r="B7" s="381" t="s">
-        <v>217</v>
+        <v>181</v>
       </c>
       <c r="C7" s="376">
         <v>4</v>
       </c>
       <c r="D7" s="393" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E7" s="394">
         <f t="shared" si="0"/>
@@ -4225,7 +4342,7 @@
         <v>25</v>
       </c>
       <c r="H7" s="387" t="s">
-        <v>165</v>
+        <v>220</v>
       </c>
       <c r="I7" s="395" t="str">
         <f t="shared" si="3"/>
@@ -4236,33 +4353,33 @@
         <v>Т789АН402</v>
       </c>
       <c r="K7" s="387" t="s">
-        <v>188</v>
-      </c>
-      <c r="L7" s="387" t="s">
-        <v>180</v>
+        <v>240</v>
+      </c>
+      <c r="L7" s="424" t="s">
+        <v>210</v>
       </c>
       <c r="M7" s="387" t="str">
         <f t="shared" si="5"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "АгроЛогистик Z7"</v>
       </c>
       <c r="N7" s="387" t="s">
-        <v>175</v>
+        <v>230</v>
       </c>
       <c r="O7" s="387" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="P7" s="387" t="str">
         <f t="shared" si="6"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "АгроЛогистик Z7"</v>
       </c>
       <c r="Q7" s="387" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="R7" s="395" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="S7" s="387" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="T7" s="387">
         <v>35980</v>
@@ -4274,20 +4391,20 @@
         <v>21660</v>
       </c>
       <c r="W7" s="387" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="X7" s="387" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="Y7" s="387" t="s">
-        <v>202</v>
+        <v>176</v>
       </c>
       <c r="Z7" s="387" t="s">
-        <v>206</v>
-      </c>
-      <c r="AA7" s="387" t="str">
+        <v>251</v>
+      </c>
+      <c r="AA7" s="428" t="str">
         <f t="shared" si="7"/>
-        <v>Водитель 4</v>
+        <v>Попович Д.О.</v>
       </c>
       <c r="AB7" s="377" t="s">
         <v>132</v>
@@ -4298,13 +4415,13 @@
         <v>45951</v>
       </c>
       <c r="B8" s="381" t="s">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="C8" s="376">
         <v>5</v>
       </c>
       <c r="D8" s="393" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E8" s="394">
         <f t="shared" si="0"/>
@@ -4319,7 +4436,7 @@
         <v>25</v>
       </c>
       <c r="H8" s="387" t="s">
-        <v>165</v>
+        <v>221</v>
       </c>
       <c r="I8" s="395" t="str">
         <f t="shared" si="3"/>
@@ -4330,33 +4447,33 @@
         <v>В321ОО599</v>
       </c>
       <c r="K8" s="387" t="s">
-        <v>188</v>
-      </c>
-      <c r="L8" s="387" t="s">
-        <v>181</v>
+        <v>241</v>
+      </c>
+      <c r="L8" s="425" t="s">
+        <v>198</v>
       </c>
       <c r="M8" s="387" t="str">
         <f t="shared" si="5"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ЮгЗерноСнаб X2"</v>
       </c>
       <c r="N8" s="387" t="s">
-        <v>175</v>
+        <v>231</v>
       </c>
       <c r="O8" s="387" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="P8" s="387" t="str">
         <f t="shared" si="6"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ЮгЗерноСнаб X2"</v>
       </c>
       <c r="Q8" s="387" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="R8" s="396" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="S8" s="387" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="T8" s="397">
         <v>32750</v>
@@ -4368,20 +4485,20 @@
         <v>16840</v>
       </c>
       <c r="W8" s="387" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="X8" s="387" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="Y8" s="387" t="s">
-        <v>202</v>
+        <v>176</v>
       </c>
       <c r="Z8" s="387" t="s">
-        <v>207</v>
-      </c>
-      <c r="AA8" s="387" t="str">
+        <v>252</v>
+      </c>
+      <c r="AA8" s="428" t="str">
         <f t="shared" si="7"/>
-        <v>Водитель 5</v>
+        <v>Моргин П.С.</v>
       </c>
       <c r="AB8" s="377" t="s">
         <v>132</v>
@@ -4392,13 +4509,13 @@
         <v>45952</v>
       </c>
       <c r="B9" s="381" t="s">
-        <v>219</v>
+        <v>183</v>
       </c>
       <c r="C9" s="376">
         <v>6</v>
       </c>
       <c r="D9" s="393" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E9" s="394">
         <f t="shared" si="0"/>
@@ -4413,7 +4530,7 @@
         <v>25</v>
       </c>
       <c r="H9" s="387" t="s">
-        <v>165</v>
+        <v>222</v>
       </c>
       <c r="I9" s="395" t="str">
         <f t="shared" si="3"/>
@@ -4424,33 +4541,33 @@
         <v>К654РМ750</v>
       </c>
       <c r="K9" s="387" t="s">
-        <v>188</v>
-      </c>
-      <c r="L9" s="387" t="s">
-        <v>182</v>
+        <v>242</v>
+      </c>
+      <c r="L9" s="425" t="s">
+        <v>199</v>
       </c>
       <c r="M9" s="387" t="str">
         <f t="shared" si="5"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ПотокАгро Q1"</v>
       </c>
       <c r="N9" s="387" t="s">
-        <v>175</v>
+        <v>232</v>
       </c>
       <c r="O9" s="387" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="P9" s="387" t="str">
         <f t="shared" si="6"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ПотокАгро Q1"</v>
       </c>
       <c r="Q9" s="387" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="R9" s="395" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="S9" s="387" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="T9" s="387">
         <v>34410</v>
@@ -4462,20 +4579,20 @@
         <v>19230</v>
       </c>
       <c r="W9" s="387" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="X9" s="387" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="Y9" s="387" t="s">
-        <v>202</v>
-      </c>
-      <c r="Z9" s="387" t="s">
-        <v>208</v>
-      </c>
-      <c r="AA9" s="387" t="str">
+        <v>176</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA9" s="428" t="str">
         <f t="shared" si="7"/>
-        <v>Водитель 6</v>
+        <v>Калевин Д.И.</v>
       </c>
       <c r="AB9" s="377" t="s">
         <v>132</v>
@@ -4486,13 +4603,13 @@
         <v>46000</v>
       </c>
       <c r="B10" s="381" t="s">
-        <v>220</v>
+        <v>184</v>
       </c>
       <c r="C10" s="376">
         <v>7</v>
       </c>
       <c r="D10" s="393" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E10" s="394">
         <f t="shared" si="0"/>
@@ -4507,7 +4624,7 @@
         <v>25</v>
       </c>
       <c r="H10" s="387" t="s">
-        <v>165</v>
+        <v>223</v>
       </c>
       <c r="I10" s="395" t="str">
         <f t="shared" si="3"/>
@@ -4518,33 +4635,33 @@
         <v>Н987НН222</v>
       </c>
       <c r="K10" s="387" t="s">
-        <v>188</v>
-      </c>
-      <c r="L10" s="387" t="s">
-        <v>183</v>
+        <v>243</v>
+      </c>
+      <c r="L10" s="425" t="s">
+        <v>200</v>
       </c>
       <c r="M10" s="387" t="str">
         <f t="shared" si="5"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ТерраГрейн 9X"</v>
       </c>
       <c r="N10" s="387" t="s">
-        <v>175</v>
+        <v>233</v>
       </c>
       <c r="O10" s="387" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="P10" s="387" t="str">
         <f t="shared" si="6"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ТерраГрейн 9X"</v>
       </c>
       <c r="Q10" s="387" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="R10" s="395" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="S10" s="387" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="T10" s="387">
         <v>35560</v>
@@ -4556,20 +4673,20 @@
         <v>20770</v>
       </c>
       <c r="W10" s="387" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="X10" s="387" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="Y10" s="387" t="s">
-        <v>202</v>
-      </c>
-      <c r="Z10" s="387" t="s">
-        <v>209</v>
-      </c>
-      <c r="AA10" s="387" t="str">
+        <v>176</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>254</v>
+      </c>
+      <c r="AA10" s="428" t="str">
         <f t="shared" si="7"/>
-        <v>Водитель 7</v>
+        <v>Родевский А.Н.</v>
       </c>
       <c r="AB10" s="377" t="s">
         <v>132</v>
@@ -4580,13 +4697,13 @@
         <v>46045</v>
       </c>
       <c r="B11" s="381" t="s">
-        <v>221</v>
+        <v>185</v>
       </c>
       <c r="C11" s="376">
         <v>8</v>
       </c>
       <c r="D11" s="393" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E11" s="394">
         <f t="shared" si="0"/>
@@ -4601,7 +4718,7 @@
         <v>26</v>
       </c>
       <c r="H11" s="387" t="s">
-        <v>165</v>
+        <v>224</v>
       </c>
       <c r="I11" s="395" t="str">
         <f t="shared" si="3"/>
@@ -4612,33 +4729,33 @@
         <v>С246ЕТ888</v>
       </c>
       <c r="K11" s="387" t="s">
-        <v>188</v>
-      </c>
-      <c r="L11" s="387" t="s">
-        <v>184</v>
+        <v>244</v>
+      </c>
+      <c r="L11" s="425" t="s">
+        <v>201</v>
       </c>
       <c r="M11" s="387" t="str">
         <f t="shared" si="5"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ФермаТрейд-Х"</v>
       </c>
       <c r="N11" s="387" t="s">
-        <v>175</v>
+        <v>234</v>
       </c>
       <c r="O11" s="387" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="P11" s="387" t="str">
         <f t="shared" si="6"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ФермаТрейд-Х"</v>
       </c>
       <c r="Q11" s="387" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="R11" s="395" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="S11" s="387" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="T11" s="387">
         <v>33280</v>
@@ -4650,20 +4767,20 @@
         <v>17820</v>
       </c>
       <c r="W11" s="387" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="X11" s="387" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="Y11" s="387" t="s">
-        <v>202</v>
-      </c>
-      <c r="Z11" s="387" t="s">
-        <v>210</v>
-      </c>
-      <c r="AA11" s="387" t="str">
+        <v>176</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>255</v>
+      </c>
+      <c r="AA11" s="428" t="str">
         <f t="shared" si="7"/>
-        <v>Водитель 8</v>
+        <v>Семиров А.В.</v>
       </c>
       <c r="AB11" s="377" t="s">
         <v>132</v>
@@ -4674,13 +4791,13 @@
         <v>46083</v>
       </c>
       <c r="B12" s="381" t="s">
-        <v>222</v>
+        <v>186</v>
       </c>
       <c r="C12" s="376">
         <v>9</v>
       </c>
       <c r="D12" s="393" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E12" s="394">
         <f t="shared" si="0"/>
@@ -4695,7 +4812,7 @@
         <v>26</v>
       </c>
       <c r="H12" s="387" t="s">
-        <v>165</v>
+        <v>225</v>
       </c>
       <c r="I12" s="395" t="str">
         <f t="shared" si="3"/>
@@ -4706,33 +4823,33 @@
         <v>Р135РТ311</v>
       </c>
       <c r="K12" s="387" t="s">
-        <v>188</v>
-      </c>
-      <c r="L12" s="387" t="s">
-        <v>185</v>
+        <v>245</v>
+      </c>
+      <c r="L12" s="425" t="s">
+        <v>202</v>
       </c>
       <c r="M12" s="387" t="str">
         <f t="shared" si="5"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ЗерноХаб 17B"</v>
       </c>
       <c r="N12" s="387" t="s">
-        <v>175</v>
+        <v>235</v>
       </c>
       <c r="O12" s="387" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="P12" s="387" t="str">
         <f t="shared" si="6"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "ЗерноХаб 17B"</v>
       </c>
       <c r="Q12" s="387" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="R12" s="395" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="S12" s="387" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="T12" s="387">
         <v>34870</v>
@@ -4744,20 +4861,20 @@
         <v>19920</v>
       </c>
       <c r="W12" s="387" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="X12" s="387" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="Y12" s="387" t="s">
-        <v>202</v>
-      </c>
-      <c r="Z12" s="387" t="s">
-        <v>211</v>
-      </c>
-      <c r="AA12" s="387" t="str">
+        <v>176</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>256</v>
+      </c>
+      <c r="AA12" s="428" t="str">
         <f t="shared" si="7"/>
-        <v>Водитель 9</v>
+        <v>Горевин М.О.</v>
       </c>
       <c r="AB12" s="377" t="s">
         <v>132</v>
@@ -4768,13 +4885,13 @@
         <v>46180</v>
       </c>
       <c r="B13" s="383" t="s">
-        <v>223</v>
+        <v>187</v>
       </c>
       <c r="C13" s="398">
         <v>10</v>
       </c>
       <c r="D13" s="399" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E13" s="400">
         <f t="shared" si="0"/>
@@ -4789,7 +4906,7 @@
         <v>26</v>
       </c>
       <c r="H13" s="401" t="s">
-        <v>165</v>
+        <v>226</v>
       </c>
       <c r="I13" s="402" t="str">
         <f>LEFT(B13,FIND(" ",B13)-1)</f>
@@ -4800,33 +4917,33 @@
         <v>У864УН049</v>
       </c>
       <c r="K13" s="401" t="s">
-        <v>188</v>
-      </c>
-      <c r="L13" s="401" t="s">
-        <v>186</v>
+        <v>246</v>
+      </c>
+      <c r="L13" s="426" t="s">
+        <v>203</v>
       </c>
       <c r="M13" s="401" t="str">
         <f t="shared" si="5"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "АгроСклад V3"</v>
       </c>
       <c r="N13" s="401" t="s">
-        <v>175</v>
+        <v>236</v>
       </c>
       <c r="O13" s="401" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="P13" s="401" t="str">
         <f t="shared" si="6"/>
-        <v>ООО "АБВ"</v>
+        <v>ООО "АгроСклад V3"</v>
       </c>
       <c r="Q13" s="401" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="R13" s="402" t="s">
+        <v>170</v>
+      </c>
+      <c r="S13" s="401" t="s">
         <v>174</v>
-      </c>
-      <c r="S13" s="401" t="s">
-        <v>190</v>
       </c>
       <c r="T13" s="401">
         <v>36240</v>
@@ -4838,20 +4955,20 @@
         <v>22110</v>
       </c>
       <c r="W13" s="401" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="X13" s="401" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="Y13" s="401" t="s">
-        <v>202</v>
+        <v>176</v>
       </c>
       <c r="Z13" s="401" t="s">
-        <v>212</v>
-      </c>
-      <c r="AA13" s="401" t="str">
+        <v>257</v>
+      </c>
+      <c r="AA13" s="429" t="str">
         <f t="shared" si="7"/>
-        <v>Водитель 10</v>
+        <v>Даневский К.А.</v>
       </c>
       <c r="AB13" s="403" t="s">
         <v>132</v>
@@ -5085,7 +5202,7 @@
       </c>
       <c r="N6" s="409" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!H2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!H2))</f>
-        <v>ООО "АБВ"</v>
+        <v>ООО "АгроФлоу X1"</v>
       </c>
       <c r="O6" s="409"/>
       <c r="P6" s="409"/>
@@ -5241,7 +5358,7 @@
       </c>
       <c r="AJ9" s="412" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!K2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!K2))</f>
-        <v>ИП ВГД</v>
+        <v>ООО "ТрансВектор X1"</v>
       </c>
       <c r="AK9" s="412"/>
       <c r="AL9" s="412"/>
@@ -5371,7 +5488,7 @@
       </c>
       <c r="K11" s="413" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!L2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!L2))</f>
-        <v>Водитель 1</v>
+        <v>Иванор Сергей Петрович</v>
       </c>
       <c r="L11" s="413"/>
       <c r="M11" s="413"/>
@@ -5554,7 +5671,7 @@
       </c>
       <c r="O13" s="414" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!M2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!M2))</f>
-        <v>ООО "АБВ"</v>
+        <v>ООО "АгроФлоу X1"</v>
       </c>
       <c r="P13" s="414"/>
       <c r="Q13" s="414"/>
@@ -5731,7 +5848,7 @@
       </c>
       <c r="L16" s="415" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!N2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!N2))</f>
-        <v>ООО "УФХ"</v>
+        <v>ООО "АгроЭкспорт X9"</v>
       </c>
       <c r="M16" s="415"/>
       <c r="N16" s="415"/>
@@ -6107,7 +6224,7 @@
       </c>
       <c r="R21" s="415" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!P2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!P2))</f>
-        <v>ООО "АБВ"</v>
+        <v>ООО "АгроФлоу X1"</v>
       </c>
       <c r="S21" s="415"/>
       <c r="T21" s="415"/>
@@ -6793,7 +6910,7 @@
       </c>
       <c r="M33" s="413" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!S2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!S2))</f>
-        <v>пшеница</v>
+        <v>пшеница 3 класса</v>
       </c>
       <c r="N33" s="413"/>
       <c r="O33" s="413"/>
@@ -7692,33 +7809,33 @@
       <c r="AP42" s="281"/>
       <c r="AQ42" s="281"/>
       <c r="AR42" s="282"/>
-      <c r="AS42" s="422"/>
-      <c r="AT42" s="423"/>
-      <c r="AU42" s="423"/>
-      <c r="AV42" s="423"/>
-      <c r="AW42" s="423"/>
-      <c r="AX42" s="423"/>
-      <c r="AY42" s="423"/>
-      <c r="AZ42" s="423"/>
-      <c r="BA42" s="423"/>
-      <c r="BB42" s="423"/>
-      <c r="BC42" s="423"/>
-      <c r="BD42" s="423"/>
-      <c r="BE42" s="423"/>
-      <c r="BF42" s="423"/>
-      <c r="BG42" s="423"/>
-      <c r="BH42" s="423"/>
-      <c r="BI42" s="423"/>
-      <c r="BJ42" s="423"/>
-      <c r="BK42" s="422"/>
-      <c r="BL42" s="423"/>
-      <c r="BM42" s="423"/>
-      <c r="BN42" s="423"/>
-      <c r="BO42" s="423"/>
-      <c r="BP42" s="423"/>
-      <c r="BQ42" s="423"/>
-      <c r="BR42" s="423"/>
-      <c r="BS42" s="423"/>
+      <c r="AS42" s="421"/>
+      <c r="AT42" s="422"/>
+      <c r="AU42" s="422"/>
+      <c r="AV42" s="422"/>
+      <c r="AW42" s="422"/>
+      <c r="AX42" s="422"/>
+      <c r="AY42" s="422"/>
+      <c r="AZ42" s="422"/>
+      <c r="BA42" s="422"/>
+      <c r="BB42" s="422"/>
+      <c r="BC42" s="422"/>
+      <c r="BD42" s="422"/>
+      <c r="BE42" s="422"/>
+      <c r="BF42" s="422"/>
+      <c r="BG42" s="422"/>
+      <c r="BH42" s="422"/>
+      <c r="BI42" s="422"/>
+      <c r="BJ42" s="422"/>
+      <c r="BK42" s="421"/>
+      <c r="BL42" s="422"/>
+      <c r="BM42" s="422"/>
+      <c r="BN42" s="422"/>
+      <c r="BO42" s="422"/>
+      <c r="BP42" s="422"/>
+      <c r="BQ42" s="422"/>
+      <c r="BR42" s="422"/>
+      <c r="BS42" s="422"/>
       <c r="BT42" s="254"/>
       <c r="BU42" s="255"/>
       <c r="BV42" s="255"/>
@@ -8700,7 +8817,7 @@
       <c r="BX55" s="228"/>
       <c r="CA55" s="413" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!X2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!X2))</f>
-        <v>Директор 1</v>
+        <v>Таргин Алексей Викторович</v>
       </c>
       <c r="CB55" s="413"/>
       <c r="CC55" s="413"/>
@@ -8961,22 +9078,22 @@
         <v>74</v>
       </c>
       <c r="G59" s="17"/>
-      <c r="H59" s="421" t="str">
+      <c r="H59" s="415" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!Y2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!Y2))</f>
         <v>кладовщик</v>
       </c>
-      <c r="I59" s="421"/>
-      <c r="J59" s="421"/>
-      <c r="K59" s="421"/>
-      <c r="L59" s="421"/>
-      <c r="M59" s="421"/>
-      <c r="N59" s="421"/>
-      <c r="O59" s="421"/>
-      <c r="P59" s="421"/>
-      <c r="Q59" s="421"/>
-      <c r="R59" s="421"/>
-      <c r="S59" s="421"/>
-      <c r="T59" s="421"/>
+      <c r="I59" s="415"/>
+      <c r="J59" s="415"/>
+      <c r="K59" s="415"/>
+      <c r="L59" s="415"/>
+      <c r="M59" s="415"/>
+      <c r="N59" s="415"/>
+      <c r="O59" s="415"/>
+      <c r="P59" s="415"/>
+      <c r="Q59" s="415"/>
+      <c r="R59" s="415"/>
+      <c r="S59" s="415"/>
+      <c r="T59" s="415"/>
       <c r="W59" s="228"/>
       <c r="X59" s="228"/>
       <c r="Y59" s="228"/>
@@ -8990,7 +9107,7 @@
       <c r="AG59" s="228"/>
       <c r="AJ59" s="413" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!Z2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!Z2))</f>
-        <v>Кладовщик 1</v>
+        <v>Сидорина М.А.</v>
       </c>
       <c r="AK59" s="413"/>
       <c r="AL59" s="413"/>
@@ -9038,7 +9155,7 @@
       <c r="CH59" s="228"/>
       <c r="CK59" s="413" t="str">
         <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!AA2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!AA2))</f>
-        <v>Водитель 1</v>
+        <v>Иванор С.П.</v>
       </c>
       <c r="CL59" s="413"/>
       <c r="CM59" s="413"/>

</xml_diff>

<commit_message>
Change formulas in template from VLOOKUP to INDEX-MATCH
</commit_message>
<xml_diff>
--- a/waybills-creation/waybills-demo.xlsx
+++ b/waybills-creation/waybills-demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alinaaleks\Downloads\GitHub\automations\waybills-creation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3683B0E0-DDE5-48C1-BEA4-619DE8D5444B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817CB87E-D55A-401F-9CDD-E13C486E882A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3864,9 +3864,7 @@
     <row r="2" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="398"/>
       <c r="B2" s="403"/>
-      <c r="C2" s="398">
-        <v>1</v>
-      </c>
+      <c r="C2" s="398"/>
       <c r="D2" s="401">
         <v>2</v>
       </c>
@@ -5090,7 +5088,7 @@
         <v>1</v>
       </c>
       <c r="BT3" s="406" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!D2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!D2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!D2), "")</f>
         <v>9512</v>
       </c>
       <c r="BU3" s="406"/>
@@ -5120,7 +5118,7 @@
         <v>3</v>
       </c>
       <c r="AI4" s="407">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!E2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!E2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!E2), "")</f>
         <v>15</v>
       </c>
       <c r="AJ4" s="407"/>
@@ -5131,7 +5129,7 @@
       </c>
       <c r="AN4" s="405"/>
       <c r="AO4" s="407" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!F2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!F2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!F2), "")</f>
         <v>сентября</v>
       </c>
       <c r="AP4" s="407"/>
@@ -5152,7 +5150,7 @@
       <c r="BC4" s="370"/>
       <c r="BD4" s="370"/>
       <c r="BE4" s="408">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!G2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!G2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!G2), "")</f>
         <v>25</v>
       </c>
       <c r="BF4" s="408"/>
@@ -5201,7 +5199,7 @@
         <v>8</v>
       </c>
       <c r="N6" s="409" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!H2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!H2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!H2), "")</f>
         <v>ООО "АгроФлоу X1"</v>
       </c>
       <c r="O6" s="409"/>
@@ -5295,7 +5293,7 @@
         <v>10</v>
       </c>
       <c r="S7" s="411" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!I2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!I2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!I2), "")</f>
         <v>КАМАЗ</v>
       </c>
       <c r="T7" s="411"/>
@@ -5315,7 +5313,7 @@
         <v>11</v>
       </c>
       <c r="BK7" s="410" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!J2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!J2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!J2), "")</f>
         <v>О975ВВ761</v>
       </c>
       <c r="BL7" s="410"/>
@@ -5357,7 +5355,7 @@
         <v>14</v>
       </c>
       <c r="AJ9" s="412" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!K2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!K2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!K2), "")</f>
         <v>ООО "ТрансВектор X1"</v>
       </c>
       <c r="AK9" s="412"/>
@@ -5487,7 +5485,7 @@
         <v>16</v>
       </c>
       <c r="K11" s="413" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!L2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!L2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!L2), "")</f>
         <v>Иванор Сергей Петрович</v>
       </c>
       <c r="L11" s="413"/>
@@ -5670,7 +5668,7 @@
         <v>21</v>
       </c>
       <c r="O13" s="414" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!M2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!M2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!M2), "")</f>
         <v>ООО "АгроФлоу X1"</v>
       </c>
       <c r="P13" s="414"/>
@@ -5847,7 +5845,7 @@
         <v>23</v>
       </c>
       <c r="L16" s="415" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!N2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!N2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!N2), "")</f>
         <v>ООО "АгроЭкспорт X9"</v>
       </c>
       <c r="M16" s="415"/>
@@ -6028,7 +6026,7 @@
         <v>25</v>
       </c>
       <c r="L18" s="415" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!O2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!O2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!O2), "")</f>
         <v>Краснодарский край</v>
       </c>
       <c r="M18" s="415"/>
@@ -6223,7 +6221,7 @@
         <v>28</v>
       </c>
       <c r="R21" s="415" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!P2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!P2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!P2), "")</f>
         <v>ООО "АгроФлоу X1"</v>
       </c>
       <c r="S21" s="415"/>
@@ -6409,7 +6407,7 @@
         <v>24</v>
       </c>
       <c r="L23" s="416" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!Q2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!Q2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!Q2), "")</f>
         <v>Ростовская обл.</v>
       </c>
       <c r="M23" s="417"/>
@@ -6691,7 +6689,7 @@
         <v>31</v>
       </c>
       <c r="AY27" s="413" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!R2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!R2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!R2), "")</f>
         <v>СК214461</v>
       </c>
       <c r="AZ27" s="413"/>
@@ -6909,7 +6907,7 @@
         <v>36</v>
       </c>
       <c r="M33" s="413" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!S2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!S2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!S2), "")</f>
         <v>пшеница 3 класса</v>
       </c>
       <c r="N33" s="413"/>
@@ -7687,7 +7685,7 @@
       <c r="AQ41" s="291"/>
       <c r="AR41" s="292"/>
       <c r="AS41" s="419">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!T2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!T2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!T2), "")</f>
         <v>34600</v>
       </c>
       <c r="AT41" s="420"/>
@@ -7699,7 +7697,7 @@
       <c r="AZ41" s="420"/>
       <c r="BA41" s="420"/>
       <c r="BB41" s="420">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!U2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!U2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!U2), "")</f>
         <v>15220</v>
       </c>
       <c r="BC41" s="420"/>
@@ -7711,7 +7709,7 @@
       <c r="BI41" s="420"/>
       <c r="BJ41" s="420"/>
       <c r="BK41" s="419">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!V2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!V2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!V2), "")</f>
         <v>19380</v>
       </c>
       <c r="BL41" s="420"/>
@@ -8757,7 +8755,7 @@
         <v>68</v>
       </c>
       <c r="S55" s="413" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!W2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!W2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!W2), "")</f>
         <v>директор</v>
       </c>
       <c r="T55" s="413"/>
@@ -8816,7 +8814,7 @@
       <c r="BW55" s="228"/>
       <c r="BX55" s="228"/>
       <c r="CA55" s="413" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!X2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!X2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!X2), "")</f>
         <v>Таргин Алексей Викторович</v>
       </c>
       <c r="CB55" s="413"/>
@@ -9079,7 +9077,7 @@
       </c>
       <c r="G59" s="17"/>
       <c r="H59" s="415" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!Y2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!Y2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!Y2), "")</f>
         <v>кладовщик</v>
       </c>
       <c r="I59" s="415"/>
@@ -9106,7 +9104,7 @@
       <c r="AF59" s="228"/>
       <c r="AG59" s="228"/>
       <c r="AJ59" s="413" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!Z2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!Z2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!Z2), "")</f>
         <v>Сидорина М.А.</v>
       </c>
       <c r="AK59" s="413"/>
@@ -9154,7 +9152,7 @@
       <c r="CG59" s="228"/>
       <c r="CH59" s="228"/>
       <c r="CK59" s="413" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!AA2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!AA2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!AA2), "")</f>
         <v>Иванор С.П.</v>
       </c>
       <c r="CL59" s="413"/>
@@ -9289,7 +9287,7 @@
         <v>77</v>
       </c>
       <c r="N61" s="413" t="str">
-        <f>IF(VLOOKUP($DE$1,свод!C:AB,свод!AB2)=0,"",VLOOKUP($DE$1,свод!C:AB,свод!AB2))</f>
+        <f>IFERROR(INDEX(свод!C:AB, MATCH($DE$1, свод!C:C, 0), свод!AB2), "")</f>
         <v>Декларация соответствия</v>
       </c>
       <c r="O61" s="413"/>

</xml_diff>